<commit_message>
Validate and repair Excel worksheet ordering and charts
</commit_message>
<xml_diff>
--- a/downloads/Instructor_Hours_Tracker_FY2027.xlsx
+++ b/downloads/Instructor_Hours_Tracker_FY2027.xlsx
@@ -529,7 +529,7 @@
       <c:legendPos val="b"/>
       <c:layout/>
     </c:legend>
-    <c:plotVisOnly val="1"/>
+    <c:plotVisOnly val="0"/>
   </c:chart>
 </c:chartSpace>
 </file>
@@ -632,7 +632,7 @@
       <c:legendPos val="r"/>
       <c:layout/>
     </c:legend>
-    <c:plotVisOnly val="1"/>
+    <c:plotVisOnly val="0"/>
   </c:chart>
 </c:chartSpace>
 </file>
@@ -789,6 +789,17 @@
         <v>0</v>
       </c>
     </row>
+    <row r="13">
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contact Hours</t>
+        </is>
+      </c>
+      <c r="R13" s="5">
+        <f>A7</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -805,6 +816,15 @@
           <t xml:space="preserve">YEAR ELAPSED</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Production Hours</t>
+        </is>
+      </c>
+      <c r="R14" s="5">
+        <f>C7</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" ht="27" customHeight="1">
       <c r="A15" s="6">
@@ -817,6 +837,15 @@
       </c>
       <c r="E15" s="7">
         <f>IF(TODAY()&lt;DATE(B4-1,10,1),0,IF(TODAY()&gt;DATE(B4,9,30),1,(TODAY()-DATE(B4-1,10,1)+1)/(DATE(B4,10,1)-DATE(B4-1,10,1))))</f>
+        <v>0</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consultation Hours</t>
+        </is>
+      </c>
+      <c r="R15" s="5">
+        <f>E7</f>
         <v>0</v>
       </c>
     </row>
@@ -911,6 +940,11 @@
         <f>IF(TODAY()&lt;A36,0,IF(TODAY()&gt;=EDATE(A36,1),1,(TODAY()-A36+1)/(EDATE(A36,1)-A36)))</f>
         <v>0</v>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oct</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="12">
@@ -937,6 +971,11 @@
         <f>IF(TODAY()&lt;A37,0,IF(TODAY()&gt;=EDATE(A37,1),1,(TODAY()-A37+1)/(EDATE(A37,1)-A37)))</f>
         <v>0</v>
       </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nov</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="12">
@@ -963,6 +1002,11 @@
         <f>IF(TODAY()&lt;A38,0,IF(TODAY()&gt;=EDATE(A38,1),1,(TODAY()-A38+1)/(EDATE(A38,1)-A38)))</f>
         <v>0</v>
       </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dec</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="12">
@@ -989,6 +1033,11 @@
         <f>IF(TODAY()&lt;A39,0,IF(TODAY()&gt;=EDATE(A39,1),1,(TODAY()-A39+1)/(EDATE(A39,1)-A39)))</f>
         <v>0</v>
       </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jan</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="12">
@@ -1015,6 +1064,11 @@
         <f>IF(TODAY()&lt;A40,0,IF(TODAY()&gt;=EDATE(A40,1),1,(TODAY()-A40+1)/(EDATE(A40,1)-A40)))</f>
         <v>0</v>
       </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feb</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="12">
@@ -1041,6 +1095,11 @@
         <f>IF(TODAY()&lt;A41,0,IF(TODAY()&gt;=EDATE(A41,1),1,(TODAY()-A41+1)/(EDATE(A41,1)-A41)))</f>
         <v>0</v>
       </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mar</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="12">
@@ -1067,6 +1126,11 @@
         <f>IF(TODAY()&lt;A42,0,IF(TODAY()&gt;=EDATE(A42,1),1,(TODAY()-A42+1)/(EDATE(A42,1)-A42)))</f>
         <v>0</v>
       </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apr</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="12">
@@ -1093,6 +1157,11 @@
         <f>IF(TODAY()&lt;A43,0,IF(TODAY()&gt;=EDATE(A43,1),1,(TODAY()-A43+1)/(EDATE(A43,1)-A43)))</f>
         <v>0</v>
       </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">May</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="12">
@@ -1119,6 +1188,11 @@
         <f>IF(TODAY()&lt;A44,0,IF(TODAY()&gt;=EDATE(A44,1),1,(TODAY()-A44+1)/(EDATE(A44,1)-A44)))</f>
         <v>0</v>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jun</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="12">
@@ -1145,6 +1219,11 @@
         <f>IF(TODAY()&lt;A45,0,IF(TODAY()&gt;=EDATE(A45,1),1,(TODAY()-A45+1)/(EDATE(A45,1)-A45)))</f>
         <v>0</v>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jul</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="12">
@@ -1171,6 +1250,11 @@
         <f>IF(TODAY()&lt;A46,0,IF(TODAY()&gt;=EDATE(A46,1),1,(TODAY()-A46+1)/(EDATE(A46,1)-A46)))</f>
         <v>0</v>
       </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aug</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="12">
@@ -1196,6 +1280,11 @@
       <c r="F47" s="7">
         <f>IF(TODAY()&lt;A47,0,IF(TODAY()&gt;=EDATE(A47,1),1,(TODAY()-A47+1)/(EDATE(A47,1)-A47)))</f>
         <v>0</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sep</t>
+        </is>
       </c>
     </row>
     <row r="48" ht="27" customHeight="1">
@@ -1232,130 +1321,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Contact Hours</t>
-        </is>
-      </c>
-      <c r="R13" s="5">
-        <f>A7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Production Hours</t>
-        </is>
-      </c>
-      <c r="R14" s="5">
-        <f>C7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Consultation Hours</t>
-        </is>
-      </c>
-      <c r="R15" s="5">
-        <f>E7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Oct</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nov</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jan</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Feb</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mar</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Apr</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">May</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jun</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jul</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Aug</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sep</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B4">
-      <formula1>2000</formula1>
-      <formula2>2100</formula2>
-    </dataValidation>
-  </dataValidations>
   <conditionalFormatting sqref="F36:F48">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
@@ -1365,6 +1331,12 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="whole" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B4">
+      <formula1>2000</formula1>
+      <formula2>2100</formula2>
+    </dataValidation>
+  </dataValidations>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>

</xml_diff>